<commit_message>
add new format to pass temporal distributions in an excel file
</commit_message>
<xml_diff>
--- a/notebooks/data/example_electric_vehicle_standalone.xlsx
+++ b/notebooks/data/example_electric_vehicle_standalone.xlsx
@@ -1,26 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vitoresearch-my.sharepoint.com/personal/amelie_muller_vito_be/Documents/Documents/04_Coding/tictac_lca/notebooks/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ajakobs/Documents/prospective_dynamic_lca/bw_timex/notebooks/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{4241AA12-71EA-40D4-81F8-7C28C4CA7D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECDB0F2E-8694-4847-A768-4E45EDD1909A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE95C60-2992-9C40-A3E4-CAF6362133F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="foreground" sheetId="2" r:id="rId1"/>
+    <sheet name="new format" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="57">
   <si>
     <t>Database</t>
   </si>
@@ -146,13 +160,58 @@
   </si>
   <si>
     <t>somewhere</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>resolution</t>
+  </si>
+  <si>
+    <t>-2,-1,0</t>
+  </si>
+  <si>
+    <t>0.7,0.1,0.2</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>timedelta64</t>
+  </si>
+  <si>
+    <t>-3,-2</t>
+  </si>
+  <si>
+    <t>2,8</t>
+  </si>
+  <si>
+    <t>0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15</t>
+  </si>
+  <si>
+    <t>delta</t>
+  </si>
+  <si>
+    <t>relative</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>y</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,6 +225,12 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -191,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -203,6 +268,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -508,7 +579,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -519,7 +590,7 @@
     <col min="8" max="8" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -527,7 +598,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -535,7 +606,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>36</v>
       </c>
@@ -543,7 +614,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -551,7 +622,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -559,7 +630,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -567,7 +638,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -575,12 +646,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -606,7 +677,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -630,7 +701,7 @@
       </c>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
@@ -656,7 +727,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -682,7 +753,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -708,7 +779,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>1</v>
       </c>
@@ -716,7 +787,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>36</v>
       </c>
@@ -724,7 +795,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -732,7 +803,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -740,7 +811,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -748,7 +819,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -756,12 +827,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>2</v>
       </c>
@@ -787,7 +858,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -811,7 +882,7 @@
       </c>
       <c r="H24" s="3"/>
     </row>
-    <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>7</v>
       </c>
@@ -837,7 +908,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
@@ -863,7 +934,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>29</v>
       </c>
@@ -889,7 +960,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>1</v>
       </c>
@@ -897,7 +968,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>36</v>
       </c>
@@ -905,7 +976,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -913,7 +984,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -921,7 +992,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -929,7 +1000,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>10</v>
       </c>
@@ -937,12 +1008,12 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>2</v>
       </c>
@@ -968,7 +1039,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>27</v>
       </c>
@@ -992,7 +1063,7 @@
       </c>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
@@ -1018,7 +1089,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>34</v>
       </c>
@@ -1044,7 +1115,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>35</v>
       </c>
@@ -1073,4 +1144,682 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FEF1186-3E2C-254B-8B01-B816012645D3}">
+  <dimension ref="A1:K40"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="90" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2">
+        <v>840</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="2">
+        <v>80</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13">
+        <v>-1</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="2">
+        <v>280</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I14">
+        <v>-1</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="3"/>
+    </row>
+    <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="2">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="2">
+        <v>-1</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I26">
+        <v>16</v>
+      </c>
+      <c r="J26">
+        <v>1</v>
+      </c>
+      <c r="K26" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="2">
+        <v>30000</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I27" t="s">
+        <v>50</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="2">
+        <v>-1</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" s="3"/>
+    </row>
+    <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="2">
+        <v>-840</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I38">
+        <v>3</v>
+      </c>
+      <c r="J38">
+        <v>1</v>
+      </c>
+      <c r="K38" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="2">
+        <v>-80</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I39">
+        <v>3</v>
+      </c>
+      <c r="J39">
+        <v>1</v>
+      </c>
+      <c r="K39" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="2">
+        <v>-280</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I40">
+        <v>3</v>
+      </c>
+      <c r="J40">
+        <v>1</v>
+      </c>
+      <c r="K40" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add easytimedelta and easy datetime options in excel reader
</commit_message>
<xml_diff>
--- a/notebooks/data/example_electric_vehicle_standalone.xlsx
+++ b/notebooks/data/example_electric_vehicle_standalone.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ajakobs/Documents/prospective_dynamic_lca/bw_timex/notebooks/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE95C60-2992-9C40-A3E4-CAF6362133F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4DD8CF2-C321-494D-8510-E6D1DF4EA6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="foreground" sheetId="2" r:id="rId1"/>
     <sheet name="new format" sheetId="3" r:id="rId2"/>
+    <sheet name="easy_tds" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="67">
   <si>
     <t>Database</t>
   </si>
@@ -205,13 +206,43 @@
   </si>
   <si>
     <t>y</t>
+  </si>
+  <si>
+    <t>easy_td</t>
+  </si>
+  <si>
+    <t>start</t>
+  </si>
+  <si>
+    <t>end</t>
+  </si>
+  <si>
+    <t>steps</t>
+  </si>
+  <si>
+    <t>td_kind</t>
+  </si>
+  <si>
+    <t>triangular</t>
+  </si>
+  <si>
+    <t>td_param</t>
+  </si>
+  <si>
+    <t>normal</t>
+  </si>
+  <si>
+    <t>easy_timedelta</t>
+  </si>
+  <si>
+    <t>easy_dt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,6 +254,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -233,6 +265,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -256,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -276,6 +314,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1280,7 +1319,7 @@
       </c>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
@@ -1315,7 +1354,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1350,7 +1389,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1822,4 +1861,720 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6DACBE-E79B-D04B-98C0-DA0BB3A15B9F}">
+  <dimension ref="A1:P40"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="90" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2">
+        <v>840</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="2">
+        <v>80</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13">
+        <v>-1</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="2">
+        <v>280</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I14">
+        <v>-1</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="P23" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="3"/>
+    </row>
+    <row r="25" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="2">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I25" s="6"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L25">
+        <v>-3</v>
+      </c>
+      <c r="M25">
+        <v>-1</v>
+      </c>
+      <c r="N25">
+        <v>3</v>
+      </c>
+      <c r="O25" t="s">
+        <v>62</v>
+      </c>
+      <c r="P25">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="2">
+        <v>-1</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="K26" t="s">
+        <v>46</v>
+      </c>
+      <c r="L26">
+        <v>14</v>
+      </c>
+      <c r="M26">
+        <v>16</v>
+      </c>
+      <c r="N26">
+        <v>3</v>
+      </c>
+      <c r="O26" t="s">
+        <v>64</v>
+      </c>
+      <c r="P26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="16" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="2">
+        <v>30000</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="7">
+        <v>45069</v>
+      </c>
+      <c r="M27" s="7">
+        <v>46165</v>
+      </c>
+      <c r="N27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="2">
+        <v>-1</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" s="3"/>
+    </row>
+    <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="2">
+        <v>-840</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I38">
+        <v>3</v>
+      </c>
+      <c r="J38">
+        <v>1</v>
+      </c>
+      <c r="K38" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="2">
+        <v>-80</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I39">
+        <v>3</v>
+      </c>
+      <c r="J39">
+        <v>1</v>
+      </c>
+      <c r="K39" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="2">
+        <v>-280</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I40">
+        <v>3</v>
+      </c>
+      <c r="J40">
+        <v>1</v>
+      </c>
+      <c r="K40" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add example notebook for excel import
</commit_message>
<xml_diff>
--- a/notebooks/data/example_electric_vehicle_standalone.xlsx
+++ b/notebooks/data/example_electric_vehicle_standalone.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -320,7 +320,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
update excel reading docs
</commit_message>
<xml_diff>
--- a/notebooks/data/example_electric_vehicle_standalone.xlsx
+++ b/notebooks/data/example_electric_vehicle_standalone.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ajakobs/Documents/prospective_dynamic_lca/bw_timex/notebooks/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F3F2AA-078C-F64C-AB79-E86FAFD9D807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3441D2-A7B3-E341-98E4-D9D5837B9911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="foreground" sheetId="2" r:id="rId1"/>
-    <sheet name="new format" sheetId="3" r:id="rId2"/>
-    <sheet name="easy_tds" sheetId="4" r:id="rId3"/>
+    <sheet name="relative_tds" sheetId="3" r:id="rId1"/>
+    <sheet name="easy_tds" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="63">
   <si>
     <t>Database</t>
   </si>
@@ -94,15 +93,9 @@
     <t>technosphere</t>
   </si>
   <si>
-    <t>{"__loader__": "bw_temporalis.TemporalDistribution", "date_dtype": "timedelta64[Y]", "date": [-2, -1, 0], "amount": [0.7, 0.1, 0.2]}</t>
-  </si>
-  <si>
     <t>powertrain</t>
   </si>
   <si>
-    <t>{"__loader__": "bw_temporalis.TemporalDistribution", "date_dtype": "timedelta64[Y]", "date": [-1], "amount": [1.0]}</t>
-  </si>
-  <si>
     <t>battery</t>
   </si>
   <si>
@@ -115,28 +108,16 @@
     <t>transport over an ev lifetime</t>
   </si>
   <si>
-    <t>{"__loader__": "bw_temporalis.TemporalDistribution", "date_dtype": "timedelta64[M]", "date": [-3, -2], "amount": [0.2, 0.8]}</t>
-  </si>
-  <si>
     <t>used electric vehicle</t>
   </si>
   <si>
-    <t>{"__loader__": "bw_temporalis.TemporalDistribution", "date_dtype": "timedelta64[Y]", "date": [16], "amount": [1.0]}</t>
-  </si>
-  <si>
     <t>electricity</t>
   </si>
   <si>
     <t>kilowatt hour</t>
   </si>
   <si>
-    <t>{"__loader__": "bw_temporalis.TemporalDistribution", "date_dtype": "timedelta64[Y]", "date": [0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15], "amount": [0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625, 0.0625]}</t>
-  </si>
-  <si>
     <t>glider_eol</t>
-  </si>
-  <si>
-    <t>{"__loader__": "bw_temporalis.TemporalDistribution", "date_dtype": "timedelta64[M]", "date": [3], "amount": [1.0]}</t>
   </si>
   <si>
     <t>powertrain_eol</t>
@@ -622,576 +603,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="90" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="2">
-        <v>1</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2">
-        <v>840</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="2">
-        <v>80</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="2">
-        <v>280</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="2">
-        <v>1</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H24" s="3"/>
-    </row>
-    <row r="25" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" s="2">
-        <v>1</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C26" s="2">
-        <v>-1</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="48" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27" s="2">
-        <v>30000</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>10</v>
-      </c>
-      <c r="B34">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C37" s="2">
-        <v>-1</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" s="3"/>
-    </row>
-    <row r="38" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C38" s="2">
-        <v>-840</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A39" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C39" s="2">
-        <v>-80</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C40" s="2">
-        <v>-280</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FEF1186-3E2C-254B-8B01-B816012645D3}">
   <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1223,10 +634,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -1247,10 +658,10 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -1280,7 +691,7 @@
         <v>4</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
@@ -1292,13 +703,13 @@
         <v>14</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
@@ -1315,7 +726,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>6</v>
@@ -1339,7 +750,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>17</v>
@@ -1348,24 +759,24 @@
         <v>18</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="K12" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="2">
         <v>80</v>
@@ -1374,7 +785,7 @@
         <v>5</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>17</v>
@@ -1383,7 +794,7 @@
         <v>18</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I13">
         <v>-1</v>
@@ -1392,15 +803,15 @@
         <v>1</v>
       </c>
       <c r="K13" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2">
         <v>280</v>
@@ -1409,7 +820,7 @@
         <v>5</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>17</v>
@@ -1418,7 +829,7 @@
         <v>18</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I14">
         <v>-1</v>
@@ -1427,7 +838,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
@@ -1435,15 +846,15 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -1451,7 +862,7 @@
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
@@ -1459,15 +870,15 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1497,7 +908,7 @@
         <v>4</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>13</v>
@@ -1509,30 +920,30 @@
         <v>14</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="2">
-        <v>1</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>6</v>
@@ -1556,7 +967,7 @@
         <v>4</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>6</v>
@@ -1565,24 +976,24 @@
         <v>18</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C26" s="2">
         <v>-1</v>
@@ -1591,7 +1002,7 @@
         <v>4</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>6</v>
@@ -1600,7 +1011,7 @@
         <v>18</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="I26">
         <v>16</v>
@@ -1609,24 +1020,24 @@
         <v>1</v>
       </c>
       <c r="K26" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C27" s="2">
         <v>30000</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>17</v>
@@ -1635,16 +1046,16 @@
         <v>18</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="I27" t="s">
+        <v>44</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K27" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -1652,15 +1063,15 @@
         <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
@@ -1668,7 +1079,7 @@
         <v>8</v>
       </c>
       <c r="B31" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
@@ -1681,10 +1092,10 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -1714,7 +1125,7 @@
         <v>4</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>13</v>
@@ -1726,21 +1137,21 @@
         <v>14</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C37" s="2">
         <v>-1</v>
@@ -1749,7 +1160,7 @@
         <v>4</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>6</v>
@@ -1761,10 +1172,10 @@
     </row>
     <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C38" s="2">
         <v>-840</v>
@@ -1773,7 +1184,7 @@
         <v>5</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>17</v>
@@ -1782,7 +1193,7 @@
         <v>18</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="I38">
         <v>3</v>
@@ -1791,15 +1202,15 @@
         <v>1</v>
       </c>
       <c r="K38" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C39" s="2">
         <v>-80</v>
@@ -1808,7 +1219,7 @@
         <v>5</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>17</v>
@@ -1817,7 +1228,7 @@
         <v>18</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="I39">
         <v>3</v>
@@ -1826,15 +1237,15 @@
         <v>1</v>
       </c>
       <c r="K39" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C40" s="2">
         <v>-280</v>
@@ -1843,7 +1254,7 @@
         <v>5</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>17</v>
@@ -1852,7 +1263,7 @@
         <v>18</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="I40">
         <v>3</v>
@@ -1861,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="K40" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1869,7 +1280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6DACBE-E79B-D04B-98C0-DA0BB3A15B9F}">
   <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1901,10 +1312,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -1925,10 +1336,10 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -1958,7 +1369,7 @@
         <v>4</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
@@ -1970,13 +1381,13 @@
         <v>14</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
@@ -1993,7 +1404,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>6</v>
@@ -2017,7 +1428,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>17</v>
@@ -2026,24 +1437,24 @@
         <v>18</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="K12" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="2">
         <v>80</v>
@@ -2052,7 +1463,7 @@
         <v>5</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>17</v>
@@ -2061,7 +1472,7 @@
         <v>18</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I13">
         <v>-1</v>
@@ -2070,15 +1481,15 @@
         <v>1</v>
       </c>
       <c r="K13" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2">
         <v>280</v>
@@ -2087,7 +1498,7 @@
         <v>5</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>17</v>
@@ -2096,7 +1507,7 @@
         <v>18</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I14">
         <v>-1</v>
@@ -2105,7 +1516,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
@@ -2113,15 +1524,15 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
@@ -2129,7 +1540,7 @@
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
@@ -2137,15 +1548,15 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
@@ -2175,7 +1586,7 @@
         <v>4</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>13</v>
@@ -2187,48 +1598,48 @@
         <v>14</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="J23" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="O23" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="K23" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O23" s="1" t="s">
+      <c r="P23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q23" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q23" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="2">
-        <v>1</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>6</v>
@@ -2252,7 +1663,7 @@
         <v>4</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>6</v>
@@ -2261,12 +1672,12 @@
         <v>18</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="I25" s="6"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="L25">
         <v>-3</v>
@@ -2278,7 +1689,7 @@
         <v>3</v>
       </c>
       <c r="O25" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="P25">
         <v>-2</v>
@@ -2286,10 +1697,10 @@
     </row>
     <row r="26" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C26" s="2">
         <v>-1</v>
@@ -2298,7 +1709,7 @@
         <v>4</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>6</v>
@@ -2307,10 +1718,10 @@
         <v>18</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="K26" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="L26">
         <v>14</v>
@@ -2322,7 +1733,7 @@
         <v>3</v>
       </c>
       <c r="O26" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="P26">
         <v>3</v>
@@ -2330,19 +1741,19 @@
     </row>
     <row r="27" spans="1:17" ht="16" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C27" s="2">
         <v>30000</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>17</v>
@@ -2351,11 +1762,11 @@
         <v>18</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="J27" s="2"/>
       <c r="K27" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="L27" s="7">
         <v>0</v>
@@ -2367,7 +1778,7 @@
         <v>16</v>
       </c>
       <c r="Q27" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
@@ -2375,15 +1786,15 @@
         <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
@@ -2391,7 +1802,7 @@
         <v>8</v>
       </c>
       <c r="B31" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
@@ -2404,10 +1815,10 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -2437,7 +1848,7 @@
         <v>4</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>13</v>
@@ -2449,21 +1860,21 @@
         <v>14</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C37" s="2">
         <v>-1</v>
@@ -2472,7 +1883,7 @@
         <v>4</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>6</v>
@@ -2484,10 +1895,10 @@
     </row>
     <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C38" s="2">
         <v>-840</v>
@@ -2496,7 +1907,7 @@
         <v>5</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>17</v>
@@ -2505,7 +1916,7 @@
         <v>18</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="I38">
         <v>3</v>
@@ -2514,15 +1925,15 @@
         <v>1</v>
       </c>
       <c r="K38" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C39" s="2">
         <v>-80</v>
@@ -2531,7 +1942,7 @@
         <v>5</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>17</v>
@@ -2540,7 +1951,7 @@
         <v>18</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="I39">
         <v>3</v>
@@ -2549,15 +1960,15 @@
         <v>1</v>
       </c>
       <c r="K39" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C40" s="2">
         <v>-280</v>
@@ -2566,7 +1977,7 @@
         <v>5</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>17</v>
@@ -2575,7 +1986,7 @@
         <v>18</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="I40">
         <v>3</v>
@@ -2584,7 +1995,7 @@
         <v>1</v>
       </c>
       <c r="K40" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>